<commit_message>
Update workflow to match actual BC endpoints and data from Route 21 pricing workflow
Rebuilt the n8n workflow after inspecting the live "Route 21 – BC Item Pricing
This Year" workflow. Uses the same BC OData endpoints (Posted_Sales_Invoice_Lines_Excel,
Posted_Sales_Invoice_Excel, Sales_Order_Excel), same auth pattern (client credentials
OAuth2), and same Company('Live-EB'). Writes to SharePoint Excel via Microsoft Graph
API instead of HubSpot. Excel template updated with matching InvoiceLines and
OpenSalesOrders sheets.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NJsArNdX6XRRhj1qrBm62L
</commit_message>
<xml_diff>
--- a/n8n-workflows/Route21_Pricing_Report.xlsx
+++ b/n8n-workflows/Route21_Pricing_Report.xlsx
@@ -7,12 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="PricingData" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="DailyLog" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="InvoiceLines" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="OpenSalesOrders" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PricingData'!$A$1:$P$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DailyLog'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'InvoiceLines'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'OpenSalesOrders'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,31 +439,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Item No.</t>
+          <t>Item No</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -473,77 +469,57 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Invoice No</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Unit Cost</t>
+          <t>Customer No</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>List Price</t>
+          <t>Customer Name</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Sales Price</t>
+          <t>Quantity</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Sales Type</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Sales Code</t>
+          <t>Amount</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Min. Quantity</t>
+          <t>Sales Order No</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>UOM</t>
+          <t>PO Number</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Price Start Date</t>
+          <t>Posting Date</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Price End Date</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Inventory</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Blocked</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Last Modified</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Report Date</t>
+          <t>Requested Delivery</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P1"/>
+  <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -558,43 +534,43 @@
   <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Report Date</t>
+          <t>Order No</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Total Rows</t>
+          <t>Customer No</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Unique Items</t>
+          <t>Customer Name</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Avg List Price</t>
+          <t>PO Number</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Blocked Items</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Requested Delivery</t>
         </is>
       </c>
     </row>

</xml_diff>